<commit_message>
Add FastAPI service, tests, CI and Render/Docker deploy config
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAhSL5eJkCXuB4mG5GtV5s
</commit_message>
<xml_diff>
--- a/output/India_Green_Finance_Tracker.xlsx
+++ b/output/India_Green_Finance_Tracker.xlsx
@@ -1260,11 +1260,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="59142782"/>
-        <c:axId val="19635579"/>
+        <c:axId val="75430726"/>
+        <c:axId val="30172502"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="59142782"/>
+        <c:axId val="75430726"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1296,7 +1296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19635579"/>
+        <c:crossAx val="30172502"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1304,7 +1304,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19635579"/>
+        <c:axId val="30172502"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1346,7 +1346,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59142782"/>
+        <c:crossAx val="75430726"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1517,11 +1517,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97144087"/>
-        <c:axId val="16147542"/>
+        <c:axId val="66434849"/>
+        <c:axId val="53227056"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97144087"/>
+        <c:axId val="66434849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1553,7 +1553,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16147542"/>
+        <c:crossAx val="53227056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1561,7 +1561,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16147542"/>
+        <c:axId val="53227056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1603,7 +1603,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97144087"/>
+        <c:crossAx val="66434849"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1768,11 +1768,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="32937056"/>
-        <c:axId val="1123301"/>
+        <c:axId val="97725551"/>
+        <c:axId val="13949197"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="32937056"/>
+        <c:axId val="97725551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1804,7 +1804,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1123301"/>
+        <c:crossAx val="13949197"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1812,7 +1812,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1123301"/>
+        <c:axId val="13949197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1854,7 +1854,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32937056"/>
+        <c:crossAx val="97725551"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>